<commit_message>
feat: review and evaluate Sheet-defined analytics formulas and action rules
</commit_message>
<xml_diff>
--- a/docs/examples/analytics/02_Marketing_ATL_BTL.xlsx
+++ b/docs/examples/analytics/02_Marketing_ATL_BTL.xlsx
@@ -10,14 +10,16 @@
     <sheet name="BACA_DULU" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Kamus_Data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Rencana_ETL" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Master_Unit" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Master_Produk" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Master_Area" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Master_Channel" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Master_Tim" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Master_Indikator" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Marketing_Data" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Action_Plan" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Formula_Analitik" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Aturan_Action_Plan" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Master_Unit" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Master_Produk" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Master_Area" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Master_Channel" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Master_Tim" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Master_Indikator" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Marketing_Data" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Action_Plan" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="REF_unit_code">'Master_Unit'!$A$2:$A$4</definedName>
@@ -26,17 +28,19 @@
     <definedName name="REF_channel_code">'Master_Channel'!$A$2:$A$5</definedName>
     <definedName name="REF_owner_team_code">'Master_Tim'!$A$2:$A$4</definedName>
     <definedName name="REF_indicator_code">'Master_Indikator'!$A$2:$A$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BACA_DULU'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BACA_DULU'!$A$1:$B$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Kamus_Data'!$A$1:$G$72</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rencana_ETL'!$A$1:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Master_Unit'!$A$1:$C$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Master_Produk'!$A$1:$D$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Master_Area'!$A$1:$C$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Master_Channel'!$A$1:$C$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Master_Tim'!$A$1:$C$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Master_Indikator'!$A$1:$F$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Marketing_Data'!$A$1:$Z$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Action_Plan'!$A$1:$W$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Rencana_ETL'!$A$1:$G$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Formula_Analitik'!$A$1:$D$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Aturan_Action_Plan'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Master_Unit'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Master_Produk'!$A$1:$D$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Master_Area'!$A$1:$C$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Master_Channel'!$A$1:$C$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Master_Tim'!$A$1:$C$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Master_Indikator'!$A$1:$F$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Marketing_Data'!$A$1:$Z$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Action_Plan'!$A$1:$W$2</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -608,7 +612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -719,7 +723,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Master_* = MASTER. Tab data/rekap/Action_Plan = NON_MASTER. BACA_DULU, Kamus_Data, Rencana_ETL = petunjuk, Dikecualikan dari ETL.</t>
+          <t>Master_* = MASTER. Tab data/rekap/Action_Plan = NON_MASTER. BACA_DULU, Kamus_Data, Rencana_ETL, Formula_Analitik, Aturan_Action_Plan = Dikecualikan dari ETL. Dua tab kontrol diimpor melalui API analytics-rules.</t>
         </is>
       </c>
     </row>
@@ -747,13 +751,481 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Formula dan aturan</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Angka persentase memakai 0..1: 50% = 0.50. Formula memakai kode metrik aplikasi, tanpa =Excel, SQL, script atau fungsi bebas. Formula dependency harus diletakkan setelah formula acuannya.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Impor aturan API</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>POST /api/v1/analytics-rules/import-sheet memakai source_id, name, product_code dan query. Lihat rules/*.json dalam ZIP atau docs/PANDUAN_ATURAN_ANALITIK.md. Preview, reviewer berbeda menyetujui expected_hash, lalu evaluate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Produk aturan</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>demo_marketing_marketing_data</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Query aturan (JSON)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>{"join_relationships": [], "metrics": ["m_qualified_leads_count_sum", "m_spend_idr_sum"], "dimensions": ["product_code", "channel_code", "area_code", "attribution_model"], "filters": [{"field": "period_start", "operator": "between", "value": ["2026-01-01", "2026-01-31"]}, {"field": "marketing_type", "operator": "eq", "value": "BTL"}], "sort": [], "time_grain": "none", "limit": 1000, "offset": 0, "visualization": null}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B11"/>
+  <autoFilter ref="A1:B15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00047857"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>owner_team_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>team_label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>unit_code</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>TEAM-CS</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Tim Layanan</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>UNIT-CS</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>TEAM-MKT</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Tim Marketing</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>UNIT-MKT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>TEAM-OPS</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Tim Operasional</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>UNIT-OPS</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C4"/>
+  <dataValidations count="2">
+    <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
+      <formula1>=REF_owner_team_code</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
+      <formula1>=REF_unit_code</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00047857"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>indicator_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>indicator_label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>measurement_unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>direction</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>aggregation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>REVENUE</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Pendapatan tercatat</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>IDR</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>HIGHER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Jumlah pendapatan tercatat pada periode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>RESOLVED</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Kasus selesai</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>CASE</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>HIGHER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>SUM</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Jumlah kasus unik selesai pada periode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>RESPONSE_HOURS</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Jam respons awal</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>HOUR</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>LOWER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Rata-rata jam respons dari sampel yang dicatat.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>SATISFACTION</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Skor kepuasan</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>SCORE_1_5</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>HIGHER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Rating sampel 1 sampai 5, bukan CSAT/NPS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>SLA_BREACH</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Rasio pelanggaran SLA</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>RATIO</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>LOWER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>RECOMPUTE_RATIO</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Keluhan melewati SLA / keluhan cohort periode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>COST_QUALIFIED_LEAD</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Biaya per qualified lead</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>IDR_PER_LEAD</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>LOWER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>RECOMPUTE_RATIO</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Spend / qualified leads yang teratribusi dan terdeduplikasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>PRODUCT_CSAT</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>CSAT produk</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>RATIO</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>HIGHER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>RECOMPUTE_RATIO</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Skor produk 4/5 dibagi respons valid pada versi survei yang sama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>SERVICE_SCORE</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Skor layanan</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>SCORE_1_5</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>HIGHER_IS_BETTER</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>AVG</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Rataan skor layanan dalam metode/sampel yang sebanding.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F9"/>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
+      <formula1>=REF_indicator_code</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <s:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <s:sheetPr>
     <s:tabColor rgb="002563EB"/>
@@ -2674,7 +3146,7 @@
 </s:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="002563EB"/>
@@ -5365,7 +5837,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -5417,73 +5889,81 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Master_Unit</t>
+          <t>Formula_Analitik</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>MASTER</t>
+          <t>EXCLUDED</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>satu baris per unit</t>
+          <t>Satu baris per kode kontrol</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>unit_code</t>
+          <t>formula_code</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Registry master</t>
+          <t>API analytics-rules</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Review definisi sebelum menambahkan metrik</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr"/>
+          <t>Review terpisah sebelum evaluate</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Tidak di-load sebagai tabel bisnis; jangan ubah header.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Master_Produk</t>
+          <t>Aturan_Action_Plan</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>MASTER</t>
+          <t>EXCLUDED</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>satu baris per produk</t>
+          <t>Satu baris per kode kontrol</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>product_code</t>
+          <t>rule_code</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Registry master</t>
+          <t>API analytics-rules</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Review definisi sebelum menambahkan metrik</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
+          <t>Review terpisah sebelum evaluate</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Tidak di-load sebagai tabel bisnis; jangan ubah header.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Master_Area</t>
+          <t>Master_Unit</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -5493,12 +5973,12 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>satu baris per area</t>
+          <t>satu baris per unit</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>area_code</t>
+          <t>unit_code</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -5516,7 +5996,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Master_Channel</t>
+          <t>Master_Produk</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -5526,12 +6006,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>satu baris per channel</t>
+          <t>satu baris per produk</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>channel_code</t>
+          <t>product_code</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5549,7 +6029,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Master_Tim</t>
+          <t>Master_Area</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -5559,12 +6039,12 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>satu baris per tim penanggung jawab</t>
+          <t>satu baris per area</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>owner_team_code</t>
+          <t>area_code</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5582,7 +6062,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Master_Indikator</t>
+          <t>Master_Channel</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -5592,12 +6072,12 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>satu baris per indikator dengan definisi dan satuan</t>
+          <t>satu baris per channel</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>indicator_code</t>
+          <t>channel_code</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5615,84 +6095,331 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Marketing_Data</t>
+          <t>Master_Tim</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>NON_MASTER</t>
+          <t>MASTER</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>satu baris per campaign channel area produk periode</t>
+          <t>satu baris per tim penanggung jawab</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>marketing_record_id</t>
+          <t>owner_team_code</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>UPSERT</t>
+          <t>Registry master</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>spend_idr:sum [IDR]; qualified_leads_count:sum [LEAD]</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>ATL/BTL adalah klasifikasi contoh; sepakati dengan bisnis. Reach antar-channel dapat overlap, bukan jangkauan unik gabungan. Rasio total harus dihitung ulang dari pembilang/penyebut, bukan AVG CPL/ROAS.</t>
-        </is>
-      </c>
+          <t>Review definisi sebelum menambahkan metrik</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Master_Indikator</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>MASTER</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>satu baris per indikator dengan definisi dan satuan</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>indicator_code</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Registry master</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Review definisi sebelum menambahkan metrik</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Marketing_Data</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>NON_MASTER</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>satu baris per campaign channel area produk periode</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>marketing_record_id</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>UPSERT</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>spend_idr:sum [IDR]; qualified_leads_count:sum [LEAD]</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>ATL/BTL adalah klasifikasi contoh; sepakati dengan bisnis. Reach antar-channel dapat overlap, bukan jangkauan unik gabungan. Rasio total harus dihitung ulang dari pembilang/penyebut, bukan AVG CPL/ROAS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Action_Plan</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>NON_MASTER</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>satu baris per tindakan yang merujuk record temuan</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>action_id</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>UPSERT</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Review definisi sebelum menambahkan metrik</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>Baseline dibekukan sesuai periode bukti; hipotesis belum terverifikasi. Nilai follow-up kosong berarti belum dievaluasi, bukan nol.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G9"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00D97706"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>formula_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>expression</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>output_unit</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>cost_qualified_lead</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>m_spend_idr_sum / m_qualified_leads_count_sum</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>IDR_PER_LEAD</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Ambang dan formula contoh; verifikasi unit, metode, grain dan target dengan pemilik bisnis.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00D97706"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>rule_code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>formula_code</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>operator</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>threshold</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>threshold_upper</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>action_description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>owner_team_code</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>due_days</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>review_cost_qualified_lead</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>cost_qualified_lead</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>gt</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>150000</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Review biaya dan atribusi BTL sebelum mengusulkan penyesuaian campaign.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>TEAM-MKT</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00047857"/>
@@ -5783,7 +6510,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00047857"/>
@@ -5875,7 +6602,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00047857"/>
@@ -5951,7 +6678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00047857"/>
@@ -6063,424 +6790,4 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00047857"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>owner_team_code</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>team_label</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>unit_code</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>TEAM-CS</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Tim Layanan</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>UNIT-CS</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>TEAM-MKT</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Tim Marketing</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>UNIT-MKT</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TEAM-OPS</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Tim Operasional</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>UNIT-OPS</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:C4"/>
-  <dataValidations count="2">
-    <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
-      <formula1>=REF_owner_team_code</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
-      <formula1>=REF_unit_code</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="00047857"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>indicator_code</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>indicator_label</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>measurement_unit</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>direction</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>aggregation</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>definition</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>REVENUE</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Pendapatan tercatat</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>IDR</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>HIGHER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>SUM</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Jumlah pendapatan tercatat pada periode.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>RESOLVED</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Kasus selesai</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>CASE</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>HIGHER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>SUM</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>Jumlah kasus unik selesai pada periode.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>RESPONSE_HOURS</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Jam respons awal</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>HOUR</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>LOWER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>AVG</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Rata-rata jam respons dari sampel yang dicatat.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>SATISFACTION</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Skor kepuasan</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>SCORE_1_5</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>HIGHER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
-        <is>
-          <t>AVG</t>
-        </is>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>Rating sampel 1 sampai 5, bukan CSAT/NPS.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>SLA_BREACH</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Rasio pelanggaran SLA</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>LOWER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>RECOMPUTE_RATIO</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>Keluhan melewati SLA / keluhan cohort periode.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>COST_QUALIFIED_LEAD</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t>Biaya per qualified lead</t>
-        </is>
-      </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>IDR_PER_LEAD</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>LOWER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>RECOMPUTE_RATIO</t>
-        </is>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
-        <is>
-          <t>Spend / qualified leads yang teratribusi dan terdeduplikasi.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>PRODUCT_CSAT</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>CSAT produk</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>RATIO</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>HIGHER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
-        <is>
-          <t>RECOMPUTE_RATIO</t>
-        </is>
-      </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>Skor produk 4/5 dibagi respons valid pada versi survei yang sama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>SERVICE_SCORE</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Skor layanan</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>SCORE_1_5</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
-        <is>
-          <t>HIGHER_IS_BETTER</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>AVG</t>
-        </is>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>Rataan skor layanan dalam metode/sampel yang sebanding.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:F9"/>
-  <dataValidations count="1">
-    <dataValidation sqref="A2:A1001" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Kode belum ada di master" error="Pilih kode rujukan yang sah; master baru harus direview sebelum dipakai." type="list">
-      <formula1>=REF_indicator_code</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-  </tableParts>
-</worksheet>
 </file>
</xml_diff>